<commit_message>
Reworking on movement logic. Now need to handle special movement and standard movement, as well as output messages. Separated food poisoning to an entirely different function, as it has unique logic.
</commit_message>
<xml_diff>
--- a/vis/map.xlsx
+++ b/vis/map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Uni\UCSC\Year 1\C_Assignment\vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6285C3B4-A67E-4AEB-A1F2-8D9D3B77C080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{32FCA2BB-E62B-4422-9ED4-626390B1E7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>Floor 1</t>
   </si>
@@ -82,6 +82,12 @@
   <si>
     <t>?dim</t>
   </si>
+  <si>
+    <t>ST_LINK</t>
+  </si>
+  <si>
+    <t>BW_LINK</t>
+  </si>
 </sst>
 </file>
 
@@ -111,7 +117,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -132,12 +138,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -168,6 +168,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -239,23 +257,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -812,7 +832,7 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
-      <c r="O8" s="15"/>
+      <c r="O8" s="13"/>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
@@ -837,26 +857,26 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="15" t="s">
+      <c r="J9" s="3"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="5"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="14"/>
+      <c r="S9" s="14"/>
+      <c r="T9" s="4"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-      <c r="W9" s="8"/>
-      <c r="X9" s="8"/>
-      <c r="Y9" s="8"/>
-      <c r="Z9" s="8"/>
-      <c r="AA9" s="8"/>
+      <c r="W9" s="6"/>
+      <c r="X9" s="6"/>
+      <c r="Y9" s="6"/>
+      <c r="Z9" s="6"/>
+      <c r="AA9" s="6"/>
     </row>
     <row r="10" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10">
@@ -869,28 +889,28 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3" t="s">
+      <c r="J10" s="3"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="5"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="14"/>
+      <c r="S10" s="14"/>
+      <c r="T10" s="4"/>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
-      <c r="W10" s="7"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9" t="s">
+      <c r="W10" s="5"/>
+      <c r="X10" s="7"/>
+      <c r="Y10" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="Z10" s="9"/>
-      <c r="AA10" s="9"/>
+      <c r="Z10" s="7"/>
+      <c r="AA10" s="7"/>
     </row>
     <row r="11" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11">
@@ -903,24 +923,24 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="5"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="14"/>
+      <c r="S11" s="14"/>
+      <c r="T11" s="4"/>
       <c r="U11" s="2"/>
-      <c r="V11" s="13"/>
-      <c r="W11" s="7"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
-      <c r="AA11" s="9"/>
+      <c r="V11" s="11"/>
+      <c r="W11" s="5"/>
+      <c r="X11" s="7"/>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="7"/>
+      <c r="AA11" s="7"/>
     </row>
     <row r="12" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12">
@@ -933,30 +953,34 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15" t="s">
+      <c r="J12" s="13"/>
+      <c r="K12" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="15" t="s">
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P12" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="T12" s="15"/>
+      <c r="T12" s="13"/>
       <c r="U12" s="2"/>
-      <c r="V12" s="13" t="s">
+      <c r="V12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="W12" s="7"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
-      <c r="AA12" s="9"/>
+      <c r="W12" s="5"/>
+      <c r="X12" s="7"/>
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="7"/>
+      <c r="AA12" s="7"/>
     </row>
     <row r="13" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G13" t="s">
@@ -1082,249 +1106,249 @@
       <c r="B17">
         <v>0</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="T17" s="10"/>
-      <c r="U17" s="10"/>
-      <c r="V17" s="10"/>
-      <c r="W17" s="10"/>
-      <c r="X17" s="10"/>
-      <c r="Y17" s="10"/>
-      <c r="Z17" s="10"/>
-      <c r="AA17" s="10"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="8"/>
+      <c r="V17" s="8"/>
+      <c r="W17" s="8"/>
+      <c r="X17" s="8"/>
+      <c r="Y17" s="8"/>
+      <c r="Z17" s="8"/>
+      <c r="AA17" s="8"/>
     </row>
     <row r="18" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>1</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="T18" s="10"/>
-      <c r="U18" s="10"/>
-      <c r="V18" s="10"/>
-      <c r="W18" s="10"/>
-      <c r="X18" s="10"/>
-      <c r="Y18" s="10"/>
-      <c r="Z18" s="10"/>
-      <c r="AA18" s="10"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+      <c r="V18" s="8"/>
+      <c r="W18" s="8"/>
+      <c r="X18" s="8"/>
+      <c r="Y18" s="8"/>
+      <c r="Z18" s="8"/>
+      <c r="AA18" s="8"/>
     </row>
     <row r="19" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>2</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="T19" s="10"/>
-      <c r="U19" s="10"/>
-      <c r="V19" s="10"/>
-      <c r="W19" s="10"/>
-      <c r="X19" s="10"/>
-      <c r="Y19" s="10"/>
-      <c r="Z19" s="10"/>
-      <c r="AA19" s="10"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="8"/>
+      <c r="V19" s="8"/>
+      <c r="W19" s="8"/>
+      <c r="X19" s="8"/>
+      <c r="Y19" s="8"/>
+      <c r="Z19" s="8"/>
+      <c r="AA19" s="8"/>
     </row>
     <row r="20" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>3</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="T20" s="10"/>
-      <c r="U20" s="10"/>
-      <c r="V20" s="10"/>
-      <c r="W20" s="10"/>
-      <c r="X20" s="10"/>
-      <c r="Y20" s="10"/>
-      <c r="Z20" s="10"/>
-      <c r="AA20" s="10"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+      <c r="V20" s="8"/>
+      <c r="W20" s="8"/>
+      <c r="X20" s="8"/>
+      <c r="Y20" s="8"/>
+      <c r="Z20" s="8"/>
+      <c r="AA20" s="8"/>
     </row>
     <row r="21" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>4</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="T21" s="10"/>
-      <c r="U21" s="10"/>
-      <c r="V21" s="10"/>
-      <c r="W21" s="10"/>
-      <c r="X21" s="10"/>
-      <c r="Y21" s="10"/>
-      <c r="Z21" s="10"/>
-      <c r="AA21" s="10"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="T21" s="8"/>
+      <c r="U21" s="8"/>
+      <c r="V21" s="8"/>
+      <c r="W21" s="8"/>
+      <c r="X21" s="8"/>
+      <c r="Y21" s="8"/>
+      <c r="Z21" s="8"/>
+      <c r="AA21" s="8"/>
     </row>
     <row r="22" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>5</v>
       </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="T22" s="10"/>
-      <c r="U22" s="10"/>
-      <c r="V22" s="10"/>
-      <c r="W22" s="10"/>
-      <c r="X22" s="10"/>
-      <c r="Y22" s="10"/>
-      <c r="Z22" s="10"/>
-      <c r="AA22" s="10"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+      <c r="V22" s="8"/>
+      <c r="W22" s="8"/>
+      <c r="X22" s="8"/>
+      <c r="Y22" s="8"/>
+      <c r="Z22" s="8"/>
+      <c r="AA22" s="8"/>
     </row>
     <row r="23" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>6</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="11"/>
-      <c r="R23" s="11"/>
-      <c r="S23" s="11"/>
-      <c r="T23" s="10"/>
-      <c r="U23" s="10"/>
-      <c r="V23" s="10"/>
-      <c r="W23" s="10"/>
-      <c r="X23" s="10"/>
-      <c r="Y23" s="10"/>
-      <c r="Z23" s="10"/>
-      <c r="AA23" s="10"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+      <c r="O23" s="9"/>
+      <c r="P23" s="9"/>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" s="9"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="8"/>
+      <c r="V23" s="8"/>
+      <c r="W23" s="8"/>
+      <c r="X23" s="8"/>
+      <c r="Y23" s="8"/>
+      <c r="Z23" s="8"/>
+      <c r="AA23" s="8"/>
     </row>
     <row r="24" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>7</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11" t="s">
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="11"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="10"/>
-      <c r="U24" s="10"/>
-      <c r="V24" s="10"/>
-      <c r="W24" s="10"/>
-      <c r="X24" s="10"/>
-      <c r="Y24" s="10"/>
-      <c r="Z24" s="10"/>
-      <c r="AA24" s="10"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
+      <c r="S24" s="9"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="8"/>
+      <c r="V24" s="8"/>
+      <c r="W24" s="8"/>
+      <c r="X24" s="8"/>
+      <c r="Y24" s="8"/>
+      <c r="Z24" s="8"/>
+      <c r="AA24" s="8"/>
     </row>
     <row r="25" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>8</v>
       </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="10"/>
-      <c r="U25" s="10"/>
-      <c r="V25" s="10"/>
-      <c r="W25" s="10"/>
-      <c r="X25" s="10"/>
-      <c r="Y25" s="10"/>
-      <c r="Z25" s="10"/>
-      <c r="AA25" s="10"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" s="9"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+      <c r="V25" s="8"/>
+      <c r="W25" s="8"/>
+      <c r="X25" s="8"/>
+      <c r="Y25" s="8"/>
+      <c r="Z25" s="8"/>
+      <c r="AA25" s="8"/>
     </row>
     <row r="26" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>9</v>
       </c>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="12"/>
-      <c r="P26" s="12"/>
-      <c r="Q26" s="12"/>
-      <c r="R26" s="12"/>
-      <c r="S26" s="12"/>
-      <c r="T26" s="10"/>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10"/>
-      <c r="W26" s="10"/>
-      <c r="X26" s="10"/>
-      <c r="Y26" s="10"/>
-      <c r="Z26" s="10"/>
-      <c r="AA26" s="10"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="8"/>
+      <c r="V26" s="8"/>
+      <c r="W26" s="8"/>
+      <c r="X26" s="8"/>
+      <c r="Y26" s="8"/>
+      <c r="Z26" s="8"/>
+      <c r="AA26" s="8"/>
     </row>
     <row r="27" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G27" t="s">
@@ -1338,7 +1362,7 @@
       </c>
     </row>
     <row r="28" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N28" s="14">
+      <c r="N28" s="12">
         <v>784</v>
       </c>
     </row>
@@ -1452,141 +1476,141 @@
       <c r="B31">
         <v>0</v>
       </c>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="10"/>
-      <c r="N31" s="10"/>
-      <c r="O31" s="10"/>
-      <c r="P31" s="10"/>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="8"/>
     </row>
     <row r="32" spans="2:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32">
         <v>1</v>
       </c>
-      <c r="K32" s="10"/>
-      <c r="L32" s="10"/>
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-      <c r="Q32" s="10"/>
-      <c r="R32" s="10"/>
-      <c r="S32" s="10"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8"/>
+      <c r="R32" s="8"/>
+      <c r="S32" s="8"/>
     </row>
     <row r="33" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33">
         <v>2</v>
       </c>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="10"/>
-      <c r="N33" s="10"/>
-      <c r="O33" s="10"/>
-      <c r="P33" s="10"/>
-      <c r="Q33" s="10"/>
-      <c r="R33" s="10"/>
-      <c r="S33" s="10"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="8"/>
+      <c r="Q33" s="8"/>
+      <c r="R33" s="8"/>
+      <c r="S33" s="8"/>
     </row>
     <row r="34" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34">
         <v>3</v>
       </c>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
-      <c r="M34" s="10"/>
-      <c r="N34" s="10"/>
-      <c r="O34" s="10"/>
-      <c r="P34" s="10"/>
-      <c r="Q34" s="10"/>
-      <c r="R34" s="10"/>
-      <c r="S34" s="10"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="8"/>
     </row>
     <row r="35" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35">
         <v>4</v>
       </c>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
-      <c r="M35" s="10"/>
-      <c r="N35" s="10"/>
-      <c r="O35" s="10"/>
-      <c r="P35" s="10"/>
-      <c r="Q35" s="10"/>
-      <c r="R35" s="10"/>
-      <c r="S35" s="10"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
     </row>
     <row r="36" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>5</v>
       </c>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
-      <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
-      <c r="O36" s="10"/>
-      <c r="P36" s="10"/>
-      <c r="Q36" s="10"/>
-      <c r="R36" s="10"/>
-      <c r="S36" s="10"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="8"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
     </row>
     <row r="37" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37">
         <v>6</v>
       </c>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
-      <c r="O37" s="10"/>
-      <c r="P37" s="10"/>
-      <c r="Q37" s="10"/>
-      <c r="R37" s="10"/>
-      <c r="S37" s="10"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="8"/>
+      <c r="R37" s="8"/>
+      <c r="S37" s="8"/>
     </row>
     <row r="38" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38">
         <v>7</v>
       </c>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
-      <c r="O38" s="10"/>
-      <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-      <c r="R38" s="10"/>
-      <c r="S38" s="10"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
+      <c r="S38" s="8"/>
     </row>
     <row r="39" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39">
         <v>8</v>
       </c>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10"/>
-      <c r="M39" s="10"/>
-      <c r="N39" s="10"/>
-      <c r="O39" s="10"/>
-      <c r="P39" s="10"/>
-      <c r="Q39" s="10"/>
-      <c r="R39" s="10"/>
-      <c r="S39" s="10"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
+      <c r="R39" s="8"/>
+      <c r="S39" s="8"/>
     </row>
     <row r="40" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40">
         <v>9</v>
       </c>
-      <c r="K40" s="10"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
-      <c r="O40" s="10"/>
-      <c r="P40" s="10"/>
-      <c r="Q40" s="10"/>
-      <c r="R40" s="10"/>
-      <c r="S40" s="10"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8"/>
+      <c r="M40" s="8"/>
+      <c r="N40" s="8"/>
+      <c r="O40" s="8"/>
+      <c r="P40" s="8"/>
+      <c r="Q40" s="8"/>
+      <c r="R40" s="8"/>
+      <c r="S40" s="8"/>
     </row>
     <row r="41" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N41" t="s">
@@ -1594,7 +1618,7 @@
       </c>
     </row>
     <row r="43" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N43" s="14">
+      <c r="N43" s="12">
         <v>360</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added a pathfinding option and functions for player decision convenince. Still need to finish FORCED and SECOND logic, consider assigning those at maze stair switch-time.
</commit_message>
<xml_diff>
--- a/vis/map.xlsx
+++ b/vis/map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Uni\UCSC\Year 1\C_Assignment\vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32FCA2BB-E62B-4422-9ED4-626390B1E7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF53F3BA-6DA2-4227-BDF5-B013CC601C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Finished some output messages, and stair-pole traversal logic (needs testing).
</commit_message>
<xml_diff>
--- a/vis/map.xlsx
+++ b/vis/map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Uni\UCSC\Year 1\C_Assignment\vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF53F3BA-6DA2-4227-BDF5-B013CC601C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{64B92874-EDCD-4864-8502-2A6D49C42DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>Floor 1</t>
   </si>
@@ -88,12 +89,15 @@
   <si>
     <t>BW_LINK</t>
   </si>
+  <si>
+    <t>LOOP_E</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,8 +120,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -189,6 +199,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -257,7 +273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -276,6 +292,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -959,7 +976,9 @@
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
-      <c r="N12" s="15"/>
+      <c r="N12" s="18" t="s">
+        <v>16</v>
+      </c>
       <c r="O12" s="16" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Uh, I think it works now
</commit_message>
<xml_diff>
--- a/vis/map.xlsx
+++ b/vis/map.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Uni\UCSC\Year 1\C_Assignment\vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64B92874-EDCD-4864-8502-2A6D49C42DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECF5F81-2564-4FE6-ADC3-16337AA4386C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>